<commit_message>
Commit updated files for Day 3.
</commit_message>
<xml_diff>
--- a/Data Analysis Project/project/reports/sales_analysis 1.xlsx
+++ b/Data Analysis Project/project/reports/sales_analysis 1.xlsx
@@ -8,23 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sc_RushilJivan_2026\Data Analysis Project\project\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A493DB98-AFF3-4460-9D97-D09F21CCA2CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1706FE8B-27AE-4D4F-9FEF-2D8314920B87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Clean Data" sheetId="1" r:id="rId1"/>
     <sheet name="Pivot Tables" sheetId="2" r:id="rId2"/>
+    <sheet name="Dashboard" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="6" r:id="rId3"/>
+    <pivotCache cacheId="5" r:id="rId4"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="33">
   <si>
     <t>transaction_id</t>
   </si>
@@ -130,7 +131,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -163,7 +164,7 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -186,16 +187,3310 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[sales_analysis 1.xlsx]Pivot Tables!Sales by Region</c:name>
+    <c:fmtId val="3"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Pivot Tables'!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Pivot Tables'!$A$2:$A$6</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>East</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>North</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>South</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>West</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Pivot Tables'!$B$2:$B$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>270000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>260500</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>225000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>148000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-1ED9-4A32-881A-4E1D0824F507}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="182"/>
+        <c:axId val="1786503327"/>
+        <c:axId val="1786501887"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1786503327"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1786501887"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1786501887"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1786503327"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[sales_analysis 1.xlsx]Pivot Tables!Monthly Revenue Trends</c:name>
+    <c:fmtId val="2"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="28575" cap="rnd">
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:ln w="28575" cap="rnd">
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Pivot Tables'!$B$20</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Pivot Tables'!$A$21:$A$25</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2024-01</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2024-02</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2024-03</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2024-04</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Pivot Tables'!$B$21:$B$25</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>160000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>200500</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>271500</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>271500</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9D1E-4D08-873A-EB1005A650B6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1193204815"/>
+        <c:axId val="1193207695"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1193204815"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1193207695"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1193207695"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1193204815"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[sales_analysis 1.xlsx]Pivot Tables!PivotTable5</c:name>
+    <c:fmtId val="4"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="ctr"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Pivot Tables'!$B$39</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-75FA-4D42-9AAE-B71F5A611635}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-75FA-4D42-9AAE-B71F5A611635}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="35000"/>
+                      <a:lumOff val="65000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:round/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Pivot Tables'!$A$40:$A$42</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Electronics</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Furniture</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Pivot Tables'!$B$40:$B$42</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>770000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>133500</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-75FA-4D42-9AAE-B71F5A611635}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="bestFit"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>15732</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>593911</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{138C8CC6-33F3-235D-649D-7CF8E3FA76C0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>603297</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>4006</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>11205</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0E6AEE68-B11C-FDFF-CADE-D8ABCB65E018}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>175858</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>593912</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>11205</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BB3DBBD2-A875-B919-8228-2AC514A0DF3C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>11206</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>11206</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>11206</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="Rectangle 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0FF21DA0-0DFC-D5F0-D186-A41CE0DD4B2B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="11206"/>
+          <a:ext cx="10903324" cy="537882"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="00B0F0"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-ZA" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Rushil Jivan" refreshedDate="46127.681375694447" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="48" xr:uid="{C69752F6-182E-478C-856F-09CCC6803248}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:J49" sheet="Sheet1"/>
+    <worksheetSource ref="A1:J49" sheet="Clean Data"/>
   </cacheSource>
   <cacheFields count="10">
     <cacheField name="transaction_id" numFmtId="0">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1001" maxValue="1050"/>
     </cacheField>
-    <cacheField name="date" numFmtId="165">
+    <cacheField name="date" numFmtId="164">
       <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2024-01-05T00:00:00" maxDate="2024-05-01T00:00:00"/>
     </cacheField>
     <cacheField name="product" numFmtId="0">
@@ -208,7 +3503,10 @@
       </sharedItems>
     </cacheField>
     <cacheField name="category" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="2">
+        <s v="Electronics"/>
+        <s v="Furniture"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="quantity" numFmtId="0">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="7"/>
@@ -259,7 +3557,7 @@
     <n v="1001"/>
     <d v="2024-01-05T00:00:00"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="2"/>
     <n v="12000"/>
     <x v="0"/>
@@ -271,7 +3569,7 @@
     <n v="1002"/>
     <d v="2024-01-07T00:00:00"/>
     <x v="1"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="5"/>
     <n v="8000"/>
     <x v="1"/>
@@ -283,7 +3581,7 @@
     <n v="1003"/>
     <d v="2024-01-10T00:00:00"/>
     <x v="2"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="3"/>
     <n v="6000"/>
     <x v="2"/>
@@ -295,7 +3593,7 @@
     <n v="1005"/>
     <d v="2024-01-20T00:00:00"/>
     <x v="3"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="2"/>
     <n v="3000"/>
     <x v="0"/>
@@ -307,7 +3605,7 @@
     <n v="1006"/>
     <d v="2024-01-22T00:00:00"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="1"/>
     <n v="12000"/>
     <x v="1"/>
@@ -319,7 +3617,7 @@
     <n v="1007"/>
     <d v="2024-01-25T00:00:00"/>
     <x v="1"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="6"/>
     <n v="8000"/>
     <x v="2"/>
@@ -331,7 +3629,7 @@
     <n v="1008"/>
     <d v="2024-01-28T00:00:00"/>
     <x v="2"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="2"/>
     <n v="6000"/>
     <x v="3"/>
@@ -343,7 +3641,7 @@
     <n v="1009"/>
     <d v="2024-02-01T00:00:00"/>
     <x v="4"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="5"/>
     <n v="1500"/>
     <x v="0"/>
@@ -355,7 +3653,7 @@
     <n v="1010"/>
     <d v="2024-02-03T00:00:00"/>
     <x v="3"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="3"/>
     <n v="3000"/>
     <x v="1"/>
@@ -367,7 +3665,7 @@
     <n v="1011"/>
     <d v="2024-02-05T00:00:00"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="2"/>
     <n v="12000"/>
     <x v="2"/>
@@ -379,7 +3677,7 @@
     <n v="1012"/>
     <d v="2024-02-07T00:00:00"/>
     <x v="1"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="4"/>
     <n v="8000"/>
     <x v="3"/>
@@ -391,7 +3689,7 @@
     <n v="1013"/>
     <d v="2024-02-10T00:00:00"/>
     <x v="2"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="3"/>
     <n v="6000"/>
     <x v="0"/>
@@ -403,7 +3701,7 @@
     <n v="1014"/>
     <d v="2024-02-12T00:00:00"/>
     <x v="4"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="6"/>
     <n v="1500"/>
     <x v="1"/>
@@ -415,7 +3713,7 @@
     <n v="1015"/>
     <d v="2024-02-15T00:00:00"/>
     <x v="3"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="2"/>
     <n v="3000"/>
     <x v="2"/>
@@ -427,7 +3725,7 @@
     <n v="1016"/>
     <d v="2024-02-18T00:00:00"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="1"/>
     <n v="12000"/>
     <x v="3"/>
@@ -439,7 +3737,7 @@
     <n v="1017"/>
     <d v="2024-02-20T00:00:00"/>
     <x v="1"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="7"/>
     <n v="8000"/>
     <x v="0"/>
@@ -451,7 +3749,7 @@
     <n v="1018"/>
     <d v="2024-02-22T00:00:00"/>
     <x v="2"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="2"/>
     <n v="6000"/>
     <x v="1"/>
@@ -463,7 +3761,7 @@
     <n v="1019"/>
     <d v="2024-02-25T00:00:00"/>
     <x v="4"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="4"/>
     <n v="1500"/>
     <x v="2"/>
@@ -475,7 +3773,7 @@
     <n v="1020"/>
     <d v="2024-02-28T00:00:00"/>
     <x v="3"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="3"/>
     <n v="3000"/>
     <x v="3"/>
@@ -487,7 +3785,7 @@
     <n v="1021"/>
     <d v="2024-03-02T00:00:00"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="2"/>
     <n v="12000"/>
     <x v="0"/>
@@ -499,7 +3797,7 @@
     <n v="1022"/>
     <d v="2024-03-04T00:00:00"/>
     <x v="1"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="5"/>
     <n v="8000"/>
     <x v="1"/>
@@ -511,7 +3809,7 @@
     <n v="1023"/>
     <d v="2024-03-06T00:00:00"/>
     <x v="2"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="3"/>
     <n v="6000"/>
     <x v="2"/>
@@ -523,7 +3821,7 @@
     <n v="1024"/>
     <d v="2024-03-08T00:00:00"/>
     <x v="4"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="4"/>
     <n v="1500"/>
     <x v="3"/>
@@ -535,7 +3833,7 @@
     <n v="1025"/>
     <d v="2024-03-10T00:00:00"/>
     <x v="3"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="2"/>
     <n v="3000"/>
     <x v="0"/>
@@ -547,7 +3845,7 @@
     <n v="1026"/>
     <d v="2024-03-12T00:00:00"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="1"/>
     <n v="12000"/>
     <x v="1"/>
@@ -559,7 +3857,7 @@
     <n v="1027"/>
     <d v="2024-03-14T00:00:00"/>
     <x v="1"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="6"/>
     <n v="8000"/>
     <x v="2"/>
@@ -571,7 +3869,7 @@
     <n v="1028"/>
     <d v="2024-03-16T00:00:00"/>
     <x v="2"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="2"/>
     <n v="6000"/>
     <x v="3"/>
@@ -583,7 +3881,7 @@
     <n v="1029"/>
     <d v="2024-03-18T00:00:00"/>
     <x v="4"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="5"/>
     <n v="1500"/>
     <x v="0"/>
@@ -595,7 +3893,7 @@
     <n v="1030"/>
     <d v="2024-03-20T00:00:00"/>
     <x v="3"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="3"/>
     <n v="3000"/>
     <x v="1"/>
@@ -607,7 +3905,7 @@
     <n v="1031"/>
     <d v="2024-03-22T00:00:00"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="2"/>
     <n v="12000"/>
     <x v="2"/>
@@ -619,7 +3917,7 @@
     <n v="1032"/>
     <d v="2024-03-24T00:00:00"/>
     <x v="1"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="4"/>
     <n v="8000"/>
     <x v="3"/>
@@ -631,7 +3929,7 @@
     <n v="1033"/>
     <d v="2024-03-26T00:00:00"/>
     <x v="2"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="3"/>
     <n v="6000"/>
     <x v="0"/>
@@ -643,7 +3941,7 @@
     <n v="1034"/>
     <d v="2024-03-28T00:00:00"/>
     <x v="4"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="6"/>
     <n v="1500"/>
     <x v="1"/>
@@ -655,7 +3953,7 @@
     <n v="1035"/>
     <d v="2024-03-30T00:00:00"/>
     <x v="3"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="2"/>
     <n v="3000"/>
     <x v="2"/>
@@ -667,7 +3965,7 @@
     <n v="1036"/>
     <d v="2024-04-02T00:00:00"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="1"/>
     <n v="12000"/>
     <x v="3"/>
@@ -679,7 +3977,7 @@
     <n v="1037"/>
     <d v="2024-04-04T00:00:00"/>
     <x v="1"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="7"/>
     <n v="8000"/>
     <x v="0"/>
@@ -691,7 +3989,7 @@
     <n v="1038"/>
     <d v="2024-04-06T00:00:00"/>
     <x v="2"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="2"/>
     <n v="6000"/>
     <x v="1"/>
@@ -703,7 +4001,7 @@
     <n v="1039"/>
     <d v="2024-04-08T00:00:00"/>
     <x v="4"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="4"/>
     <n v="1500"/>
     <x v="2"/>
@@ -715,7 +4013,7 @@
     <n v="1040"/>
     <d v="2024-04-10T00:00:00"/>
     <x v="3"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="3"/>
     <n v="3000"/>
     <x v="3"/>
@@ -727,7 +4025,7 @@
     <n v="1041"/>
     <d v="2024-04-12T00:00:00"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="2"/>
     <n v="12000"/>
     <x v="0"/>
@@ -739,7 +4037,7 @@
     <n v="1042"/>
     <d v="2024-04-14T00:00:00"/>
     <x v="1"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="5"/>
     <n v="8000"/>
     <x v="1"/>
@@ -751,7 +4049,7 @@
     <n v="1043"/>
     <d v="2024-04-16T00:00:00"/>
     <x v="2"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="3"/>
     <n v="6000"/>
     <x v="2"/>
@@ -763,7 +4061,7 @@
     <n v="1045"/>
     <d v="2024-04-20T00:00:00"/>
     <x v="3"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="2"/>
     <n v="3000"/>
     <x v="0"/>
@@ -775,7 +4073,7 @@
     <n v="1046"/>
     <d v="2024-04-22T00:00:00"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="1"/>
     <n v="12000"/>
     <x v="1"/>
@@ -787,7 +4085,7 @@
     <n v="1047"/>
     <d v="2024-04-24T00:00:00"/>
     <x v="1"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="6"/>
     <n v="8000"/>
     <x v="2"/>
@@ -799,7 +4097,7 @@
     <n v="1048"/>
     <d v="2024-04-26T00:00:00"/>
     <x v="2"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <n v="2"/>
     <n v="6000"/>
     <x v="3"/>
@@ -811,7 +4109,7 @@
     <n v="1049"/>
     <d v="2024-04-28T00:00:00"/>
     <x v="4"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="5"/>
     <n v="1500"/>
     <x v="0"/>
@@ -823,7 +4121,7 @@
     <n v="1050"/>
     <d v="2024-04-30T00:00:00"/>
     <x v="3"/>
-    <s v="Furniture"/>
+    <x v="1"/>
     <n v="3"/>
     <n v="3000"/>
     <x v="1"/>
@@ -835,24 +4133,113 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{406183F9-9921-461D-B8CD-64696A368A07}" name="PivotTable4" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A29:B35" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B91F56DB-EC1E-48E3-8F19-69CEF914C3D2}" name="PivotTable5" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+  <location ref="A39:B42" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
-    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="4"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of revenue" fld="8" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="3">
+    <chartFormat chart="4" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="2">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="3" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="3">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="3" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A6DC9210-722F-4976-A90F-745F1129A3FE}" name="Salesperson Performance" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A29:B35" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
       <items count="6">
         <item x="2"/>
@@ -907,35 +4294,18 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CDA2139E-3EF1-4D1D-A972-EDA4720009C6}" name="PivotTable3" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{15DBC393-6459-4A9A-AE10-F83D49575CF6}" name="Monthly Revenue Trends" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
   <location ref="A20:B25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
-    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
       <items count="5">
@@ -973,6 +4343,17 @@
   <dataFields count="1">
     <dataField name="Sum of revenue" fld="8" baseField="0" baseItem="0"/>
   </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -985,12 +4366,12 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{16AB774E-8DF0-4693-A873-D67F9776C27D}" name="PivotTable2" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70B326EE-CA16-4AFF-9F76-235CAEFC87B3}" name="Top performing Products" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A10:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
-    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
       <items count="6">
         <item x="4"/>
@@ -1004,15 +4385,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
+    <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
@@ -1058,12 +4431,12 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5E186B43-97B2-46B5-878A-78523C8A65F4}" name="PivotTable1" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5E186B43-97B2-46B5-878A-78523C8A65F4}" name="Sales by Region" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12">
   <location ref="A1:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
-    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -1107,6 +4480,53 @@
   <dataFields count="1">
     <dataField name="Sum of revenue" fld="8" baseField="0" baseItem="0"/>
   </dataFields>
+  <chartFormats count="4">
+    <chartFormat chart="3" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -1406,6 +4826,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -2982,11 +6414,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FAD743A-8513-455B-83F4-D866E93A6E9D}">
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -3197,7 +6635,49 @@
         <v>903500</v>
       </c>
     </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B39" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B40" s="4">
+        <v>770000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B41" s="4">
+        <v>133500</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B42" s="4">
+        <v>903500</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD5186C-5331-4579-84EF-751413196B48}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>